<commit_message>
Rimossa card Progetto Scuole ridondante
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/tabella_aggiornamento_articoli.xlsx
+++ b/AppLogSolutionLocale/dati/tabella_aggiornamento_articoli.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\App\AppLogSolutionLocale\dati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA795717-8B57-409A-A735-4DFF177DCC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2675579D-E585-4A04-A50A-DD474DDAC06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4968" yWindow="2100" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Articoli" sheetId="1" r:id="rId1"/>
@@ -774,7 +774,7 @@
     <col min="2" max="2" width="47.88671875" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="6" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="8" width="14" style="3" customWidth="1"/>

</xml_diff>